<commit_message>
Solve No. of Islands
</commit_message>
<xml_diff>
--- a/DSA patterns Cheat Sheet.xlsx
+++ b/DSA patterns Cheat Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB77959-D6B2-4519-84E4-ACA7A8A45998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF9ADA1-814C-475C-8705-6DECC1E495C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3318,7 +3318,7 @@
       <c r="E124" s="8"/>
     </row>
     <row r="125" spans="1:5" ht="14.4">
-      <c r="A125" s="6"/>
+      <c r="A125" s="33"/>
       <c r="B125" s="9" t="s">
         <v>243</v>
       </c>
@@ -3331,7 +3331,7 @@
       <c r="E125" s="8"/>
     </row>
     <row r="126" spans="1:5" ht="14.4">
-      <c r="A126" s="6"/>
+      <c r="A126" s="33"/>
       <c r="B126" s="9" t="s">
         <v>246</v>
       </c>
@@ -3344,7 +3344,7 @@
       <c r="E126" s="8"/>
     </row>
     <row r="127" spans="1:5" ht="14.4">
-      <c r="A127" s="6"/>
+      <c r="A127" s="33"/>
       <c r="B127" s="9" t="s">
         <v>248</v>
       </c>
@@ -3357,7 +3357,7 @@
       <c r="E127" s="8"/>
     </row>
     <row r="128" spans="1:5" ht="14.4">
-      <c r="A128" s="6"/>
+      <c r="A128" s="33"/>
       <c r="B128" s="9" t="s">
         <v>251</v>
       </c>
@@ -3370,7 +3370,7 @@
       <c r="E128" s="8"/>
     </row>
     <row r="129" spans="1:5" ht="14.4">
-      <c r="A129" s="6"/>
+      <c r="A129" s="33"/>
       <c r="B129" s="9" t="s">
         <v>253</v>
       </c>
@@ -3383,7 +3383,7 @@
       <c r="E129" s="8"/>
     </row>
     <row r="130" spans="1:5" ht="14.4">
-      <c r="A130" s="6"/>
+      <c r="A130" s="33"/>
       <c r="B130" s="9" t="s">
         <v>255</v>
       </c>
@@ -3394,7 +3394,7 @@
       <c r="E130" s="8"/>
     </row>
     <row r="131" spans="1:5" ht="14.4">
-      <c r="A131" s="6"/>
+      <c r="A131" s="33"/>
       <c r="B131" s="9" t="s">
         <v>257</v>
       </c>
@@ -3407,7 +3407,7 @@
       <c r="E131" s="8"/>
     </row>
     <row r="132" spans="1:5" ht="14.4">
-      <c r="A132" s="6"/>
+      <c r="A132" s="33"/>
       <c r="B132" s="9" t="s">
         <v>260</v>
       </c>
@@ -3418,7 +3418,7 @@
       <c r="E132" s="8"/>
     </row>
     <row r="133" spans="1:5" ht="14.4">
-      <c r="A133" s="6"/>
+      <c r="A133" s="33"/>
       <c r="B133" s="9" t="s">
         <v>262</v>
       </c>
@@ -3559,7 +3559,7 @@
       </c>
     </row>
     <row r="148" spans="1:3" ht="13.2">
-      <c r="B148" s="18" t="s">
+      <c r="B148" s="34" t="s">
         <v>295</v>
       </c>
       <c r="C148" s="29" t="s">
@@ -3567,7 +3567,7 @@
       </c>
     </row>
     <row r="149" spans="1:3" ht="13.2">
-      <c r="B149" s="18" t="s">
+      <c r="B149" s="34" t="s">
         <v>297</v>
       </c>
       <c r="C149" s="29" t="s">
@@ -3602,7 +3602,7 @@
       <c r="A153" s="30" t="s">
         <v>305</v>
       </c>
-      <c r="B153" s="18" t="s">
+      <c r="B153" s="34" t="s">
         <v>306</v>
       </c>
       <c r="C153" s="29" t="s">
@@ -3610,7 +3610,7 @@
       </c>
     </row>
     <row r="154" spans="1:3" ht="13.2">
-      <c r="B154" s="18" t="s">
+      <c r="B154" s="34" t="s">
         <v>308</v>
       </c>
       <c r="C154" s="29" t="s">
@@ -3626,7 +3626,7 @@
       </c>
     </row>
     <row r="156" spans="1:3" ht="13.2">
-      <c r="B156" s="18" t="s">
+      <c r="B156" s="34" t="s">
         <v>312</v>
       </c>
       <c r="C156" s="29" t="s">
@@ -3661,7 +3661,7 @@
       <c r="A160" s="30" t="s">
         <v>320</v>
       </c>
-      <c r="B160" s="18" t="s">
+      <c r="B160" s="34" t="s">
         <v>321</v>
       </c>
       <c r="C160" s="29" t="s">
@@ -3669,7 +3669,7 @@
       </c>
     </row>
     <row r="161" spans="1:3" ht="13.2">
-      <c r="B161" s="18" t="s">
+      <c r="B161" s="34" t="s">
         <v>323</v>
       </c>
       <c r="C161" s="29" t="s">

</xml_diff>